<commit_message>
Hand check of the minimum fault current (symmetrical components + superposition)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DSDR_Study/results/database/Minimum_Fault_Current_Calculation.xlsx
+++ b/DSDR_Study/results/database/Minimum_Fault_Current_Calculation.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LG_3ohm_faults" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="If_min_R1_R2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All_sections" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hand_check" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +40,10 @@
     </font>
     <font>
       <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="4">
@@ -85,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -110,6 +115,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2797,4 +2803,299 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Hand calculation of If,min: LG fault through Rf = 3 ohm at node 680, phase B, DG out of service</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Values</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Result (hand)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>PowerFactory</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>1  Thevenin sequence impedances at 680</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Z1, Z2, Z0 seen from the fault (PowerFactory, DG out)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Z1 = Z2 = 0.2860 + j0.8161 ohm;  Z0 = 0.8014 + j2.1366 ohm</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2  Pre-fault voltage, phase B at 680</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>V_B from the load flow (complete method keeps it)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>2575.2 V at -154.95 deg (1.072 pu; regulator boost)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>3  Total loop impedance</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Z = Z1 + Z2 + Z0 + 3 Rf</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>1.3733 + j3.7688 + 9</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>10.373 + j3.769 = 11.037 ohm at 20.0 deg</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>4  Fault current at 680 (LG)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>I_f = 3 V_B / (Z1 + Z2 + Z0 + 3 Rf)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>3 x 2575.2 / 11.037</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>700.0 A at -174.9 deg</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>701.5 A at -176.0 deg</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>-0.2 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>5  Load current through R2, phase B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>from the load flow (before the fault)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>184.0 A at -164.2 deg</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>6  Current through R2, phase B, during the fault</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>I_R2 = I_load,R2 + I_f   (superposition; the feeder is radial, so all of I_f passes R2)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>184.0 A at -164.2 deg + 701.5 A at -176.0 deg</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>882.5 A at -173.5 deg</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>878.5 A</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>+0.5 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>7  Load current through R1, phase B</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>from the load flow (before the fault)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>411.3 A at -173.5 deg</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>8  Current through R1, phase B, during the fault</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>I_R1 = I_load,R1 + I_f   (all of I_f also passes R1)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>411.3 A at -173.5 deg + 701.5 A at -176.0 deg</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>1112.5 A at -175.0 deg</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>1074.4 A</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>+3.5 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Why phase B gives the minimum: phase B carries the smallest load current at R1 (411 A, against 558 A on phase A and 588 A on phase C), so load + fault current is smallest on phase B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Why the R1 hand value is about 3.5 % high: superposition with the PRE-FAULT load current assumes the loads keep drawing the same current. During the fault the phase-B voltage sags, the loads supplied through R1 draw less, and PowerFactory's complete method includes that. R1 feeds more load (632, 633, 645, 646, DL and the R2 zone) than R2, so the effect is larger at R1; at R2 the hand value is within 0.5 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Result: the hand calculation confirms the PowerFactory values If,min(R1) = 1074 A and If,min(R2) = 879 A within the accuracy of superposition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Note: the R2 value is 878.5 A (rounded 879 A).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
If,min workbook: farthest node of the R1 and R2 zones from the model's line lengths
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DSDR_Study/results/database/Minimum_Fault_Current_Calculation.xlsx
+++ b/DSDR_Study/results/database/Minimum_Fault_Current_Calculation.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LG_3ohm_faults" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="If_min_R1_R2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All_sections" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hand_check" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Farthest_node" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hand_check" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -90,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -116,6 +117,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2811,6 +2815,499 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Farthest node of each recloser zone, and where the minimum fault current really is (DG out)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Node (zone of R1)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Line length from RG60 (R1, feeder head) (ft)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Fault current at the node, lowest phase (A)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Current through R1, lowest phase (A)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>632</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>739.2</v>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>1149.9 (phase B)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>633</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>718.3</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>1125.1 (phase B)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>645</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>705.5</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>1109.8 (phase B)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>646</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2800</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>686.2</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>1090.1 (phase B)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>DL</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>3010</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>697.1</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>1125.1 (phase B)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>671</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>658.8</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>1101.6 (phase B)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>692</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>658.8</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>1101.6 (phase B)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>684</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>4300</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>640.3</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>1134.1 (phase A)</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>675</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4500</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>640.4</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>1085.4 (phase B)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>611</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>622.7</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>1141.7 (phase C)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>680</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>635.5</v>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>1074.4 (phase B)</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>lowest recloser current = If,min</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>652</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>5100</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>617.2</v>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>1102.4 (phase A)</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>farthest node</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Node (zone of R2)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Line length from 671 end of line 632-671 (R2) (ft)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Fault current at the node, lowest phase (A)</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Current through R2, lowest phase (A)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>671</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>658.8</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>907.4 (phase B)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>692</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>658.8</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>907.4 (phase B)</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>684</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>640.3</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>1013.0 (phase C)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>675</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>640.4</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>890.3 (phase B)</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>611</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>600</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>622.7</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>994.8 (phase C)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>680</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>635.5</v>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>878.5 (phase B)</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>lowest recloser current = If,min</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>652</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C25" s="11" t="n">
+        <v>617.2</v>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>1028.3 (phase A)</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>farthest node</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Farthest node: largest line length from the recloser to a node of its zone, from the line lengths of the PowerFactory model (feet). R1: from RG60 at the feeder head; R2: from its position at the 671 end of line 632-671.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>R1: 650-632 2000 + 632-671 2000 + 671-684 300 + 684-652 800 = 5100 ft to node 652.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>R2: 671-684 300 + 684-652 800 = 1100 ft to node 652.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>The method takes If,min as the LG fault through 3 ohm at the farthest node (652). Because the recloser also carries the load current of its phase, the lowest recloser current is found at 680 (phase B): 1074.4 A at R1 and 878.5 A at R2. The pickups are checked against these lowest values, which is the safer choice.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A31:E31"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>